<commit_message>
Toegevoegd gegevens 'Een actueel beeld van de kans op extreme neerslag STOWA 2019 tabel 1 p.5'
</commit_message>
<xml_diff>
--- a/data-raw/xlsx/Extreme_buien.xlsx
+++ b/data-raw/xlsx/Extreme_buien.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7fa01722dbc575f3/Documenten/myR_on_GitHub/packages/scsnl/data-raw/xlsx/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="455" documentId="11_F25DC773A252ABDACC1048C0A9997A6A5ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0229C3C1-67B8-4D82-AED0-7E9271F82C98}"/>
+  <xr:revisionPtr revIDLastSave="531" documentId="11_F25DC773A252ABDACC1048C0A9997A6A5ADE58F0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{65542F6A-4291-40C7-AB0F-552C1B07EF98}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2244" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2820" uniqueCount="22">
   <si>
     <t>Q</t>
   </si>
@@ -93,6 +93,15 @@
   </si>
   <si>
     <t>Neerslagstatistiek KNMI23 tabel 11 p. 27</t>
+  </si>
+  <si>
+    <t>Een actueel beeld van de kans op extreme neerslag STOWA 2019 tabel 1 p.5</t>
+  </si>
+  <si>
+    <t>5 prct waarde</t>
+  </si>
+  <si>
+    <t>95 prct waarde</t>
   </si>
 </sst>
 </file>
@@ -424,11 +433,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J651"/>
+  <dimension ref="A1:J795"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="1"/>
     <col min="5" max="5" width="41.21875" customWidth="1"/>
+    <col min="8" max="8" width="12.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
@@ -16311,6 +16321,3766 @@
       </c>
       <c r="H651" t="s">
         <v>12</v>
+      </c>
+    </row>
+    <row r="652" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A652" s="1">
+        <v>2</v>
+      </c>
+      <c r="B652">
+        <v>10</v>
+      </c>
+      <c r="C652" t="s">
+        <v>11</v>
+      </c>
+      <c r="D652">
+        <v>8</v>
+      </c>
+      <c r="E652" t="s">
+        <v>19</v>
+      </c>
+      <c r="F652" t="s">
+        <v>9</v>
+      </c>
+      <c r="G652">
+        <v>2019</v>
+      </c>
+      <c r="H652" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="653" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A653" s="1">
+        <v>2</v>
+      </c>
+      <c r="B653">
+        <v>30</v>
+      </c>
+      <c r="C653" t="s">
+        <v>11</v>
+      </c>
+      <c r="D653">
+        <v>10</v>
+      </c>
+      <c r="E653" t="s">
+        <v>19</v>
+      </c>
+      <c r="F653" t="s">
+        <v>9</v>
+      </c>
+      <c r="G653">
+        <v>2019</v>
+      </c>
+      <c r="H653" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="654" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A654" s="1">
+        <v>2</v>
+      </c>
+      <c r="B654">
+        <v>60</v>
+      </c>
+      <c r="C654" t="s">
+        <v>11</v>
+      </c>
+      <c r="D654">
+        <v>13</v>
+      </c>
+      <c r="E654" t="s">
+        <v>19</v>
+      </c>
+      <c r="F654" t="s">
+        <v>9</v>
+      </c>
+      <c r="G654">
+        <v>2019</v>
+      </c>
+      <c r="H654" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="655" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A655" s="1">
+        <v>2</v>
+      </c>
+      <c r="B655">
+        <v>4</v>
+      </c>
+      <c r="C655" t="s">
+        <v>8</v>
+      </c>
+      <c r="D655">
+        <v>19</v>
+      </c>
+      <c r="E655" t="s">
+        <v>19</v>
+      </c>
+      <c r="F655" t="s">
+        <v>9</v>
+      </c>
+      <c r="G655">
+        <v>2019</v>
+      </c>
+      <c r="H655" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="656" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A656" s="1">
+        <v>2</v>
+      </c>
+      <c r="B656">
+        <v>12</v>
+      </c>
+      <c r="C656" t="s">
+        <v>8</v>
+      </c>
+      <c r="D656">
+        <v>25</v>
+      </c>
+      <c r="E656" t="s">
+        <v>19</v>
+      </c>
+      <c r="F656" t="s">
+        <v>9</v>
+      </c>
+      <c r="G656">
+        <v>2019</v>
+      </c>
+      <c r="H656" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="657" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A657" s="1">
+        <v>2</v>
+      </c>
+      <c r="B657">
+        <v>24</v>
+      </c>
+      <c r="C657" t="s">
+        <v>8</v>
+      </c>
+      <c r="D657">
+        <v>30</v>
+      </c>
+      <c r="E657" t="s">
+        <v>19</v>
+      </c>
+      <c r="F657" t="s">
+        <v>9</v>
+      </c>
+      <c r="G657">
+        <v>2019</v>
+      </c>
+      <c r="H657" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="658" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A658" s="1">
+        <v>2</v>
+      </c>
+      <c r="B658">
+        <v>4</v>
+      </c>
+      <c r="C658" t="s">
+        <v>14</v>
+      </c>
+      <c r="D658">
+        <v>50</v>
+      </c>
+      <c r="E658" t="s">
+        <v>19</v>
+      </c>
+      <c r="F658" t="s">
+        <v>9</v>
+      </c>
+      <c r="G658">
+        <v>2019</v>
+      </c>
+      <c r="H658" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="659" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A659" s="1">
+        <v>2</v>
+      </c>
+      <c r="B659">
+        <v>8</v>
+      </c>
+      <c r="C659" t="s">
+        <v>14</v>
+      </c>
+      <c r="D659">
+        <v>68</v>
+      </c>
+      <c r="E659" t="s">
+        <v>19</v>
+      </c>
+      <c r="F659" t="s">
+        <v>9</v>
+      </c>
+      <c r="G659">
+        <v>2019</v>
+      </c>
+      <c r="H659" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="660" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A660" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B660">
+        <v>10</v>
+      </c>
+      <c r="C660" t="s">
+        <v>11</v>
+      </c>
+      <c r="D660">
+        <v>12</v>
+      </c>
+      <c r="E660" t="s">
+        <v>19</v>
+      </c>
+      <c r="F660" t="s">
+        <v>9</v>
+      </c>
+      <c r="G660">
+        <v>2019</v>
+      </c>
+      <c r="H660" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="661" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A661" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B661">
+        <v>30</v>
+      </c>
+      <c r="C661" t="s">
+        <v>11</v>
+      </c>
+      <c r="D661">
+        <v>17</v>
+      </c>
+      <c r="E661" t="s">
+        <v>19</v>
+      </c>
+      <c r="F661" t="s">
+        <v>9</v>
+      </c>
+      <c r="G661">
+        <v>2019</v>
+      </c>
+      <c r="H661" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="662" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A662" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B662">
+        <v>60</v>
+      </c>
+      <c r="C662" t="s">
+        <v>11</v>
+      </c>
+      <c r="D662">
+        <v>20</v>
+      </c>
+      <c r="E662" t="s">
+        <v>19</v>
+      </c>
+      <c r="F662" t="s">
+        <v>9</v>
+      </c>
+      <c r="G662">
+        <v>2019</v>
+      </c>
+      <c r="H662" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="663" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A663" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B663">
+        <v>4</v>
+      </c>
+      <c r="C663" t="s">
+        <v>8</v>
+      </c>
+      <c r="D663">
+        <v>28</v>
+      </c>
+      <c r="E663" t="s">
+        <v>19</v>
+      </c>
+      <c r="F663" t="s">
+        <v>9</v>
+      </c>
+      <c r="G663">
+        <v>2019</v>
+      </c>
+      <c r="H663" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="664" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A664" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B664">
+        <v>12</v>
+      </c>
+      <c r="C664" t="s">
+        <v>8</v>
+      </c>
+      <c r="D664">
+        <v>37</v>
+      </c>
+      <c r="E664" t="s">
+        <v>19</v>
+      </c>
+      <c r="F664" t="s">
+        <v>9</v>
+      </c>
+      <c r="G664">
+        <v>2019</v>
+      </c>
+      <c r="H664" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="665" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A665" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B665">
+        <v>24</v>
+      </c>
+      <c r="C665" t="s">
+        <v>8</v>
+      </c>
+      <c r="D665">
+        <v>44</v>
+      </c>
+      <c r="E665" t="s">
+        <v>19</v>
+      </c>
+      <c r="F665" t="s">
+        <v>9</v>
+      </c>
+      <c r="G665">
+        <v>2019</v>
+      </c>
+      <c r="H665" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="666" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A666" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B666">
+        <v>4</v>
+      </c>
+      <c r="C666" t="s">
+        <v>14</v>
+      </c>
+      <c r="D666">
+        <v>69</v>
+      </c>
+      <c r="E666" t="s">
+        <v>19</v>
+      </c>
+      <c r="F666" t="s">
+        <v>9</v>
+      </c>
+      <c r="G666">
+        <v>2019</v>
+      </c>
+      <c r="H666" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="667" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A667" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B667">
+        <v>8</v>
+      </c>
+      <c r="C667" t="s">
+        <v>14</v>
+      </c>
+      <c r="D667">
+        <v>91</v>
+      </c>
+      <c r="E667" t="s">
+        <v>19</v>
+      </c>
+      <c r="F667" t="s">
+        <v>9</v>
+      </c>
+      <c r="G667">
+        <v>2019</v>
+      </c>
+      <c r="H667" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="668" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A668" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B668">
+        <v>10</v>
+      </c>
+      <c r="C668" t="s">
+        <v>11</v>
+      </c>
+      <c r="D668">
+        <v>17</v>
+      </c>
+      <c r="E668" t="s">
+        <v>19</v>
+      </c>
+      <c r="F668" t="s">
+        <v>9</v>
+      </c>
+      <c r="G668">
+        <v>2019</v>
+      </c>
+      <c r="H668" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="669" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A669" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B669">
+        <v>30</v>
+      </c>
+      <c r="C669" t="s">
+        <v>11</v>
+      </c>
+      <c r="D669">
+        <v>24</v>
+      </c>
+      <c r="E669" t="s">
+        <v>19</v>
+      </c>
+      <c r="F669" t="s">
+        <v>9</v>
+      </c>
+      <c r="G669">
+        <v>2019</v>
+      </c>
+      <c r="H669" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="670" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A670" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B670">
+        <v>60</v>
+      </c>
+      <c r="C670" t="s">
+        <v>11</v>
+      </c>
+      <c r="D670">
+        <v>30</v>
+      </c>
+      <c r="E670" t="s">
+        <v>19</v>
+      </c>
+      <c r="F670" t="s">
+        <v>9</v>
+      </c>
+      <c r="G670">
+        <v>2019</v>
+      </c>
+      <c r="H670" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="671" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A671" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B671">
+        <v>4</v>
+      </c>
+      <c r="C671" t="s">
+        <v>8</v>
+      </c>
+      <c r="D671">
+        <v>41</v>
+      </c>
+      <c r="E671" t="s">
+        <v>19</v>
+      </c>
+      <c r="F671" t="s">
+        <v>9</v>
+      </c>
+      <c r="G671">
+        <v>2019</v>
+      </c>
+      <c r="H671" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="672" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A672" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B672">
+        <v>12</v>
+      </c>
+      <c r="C672" t="s">
+        <v>8</v>
+      </c>
+      <c r="D672">
+        <v>51</v>
+      </c>
+      <c r="E672" t="s">
+        <v>19</v>
+      </c>
+      <c r="F672" t="s">
+        <v>9</v>
+      </c>
+      <c r="G672">
+        <v>2019</v>
+      </c>
+      <c r="H672" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="673" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A673" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B673">
+        <v>24</v>
+      </c>
+      <c r="C673" t="s">
+        <v>8</v>
+      </c>
+      <c r="D673">
+        <v>60</v>
+      </c>
+      <c r="E673" t="s">
+        <v>19</v>
+      </c>
+      <c r="F673" t="s">
+        <v>9</v>
+      </c>
+      <c r="G673">
+        <v>2019</v>
+      </c>
+      <c r="H673" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="674" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A674" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B674">
+        <v>4</v>
+      </c>
+      <c r="C674" t="s">
+        <v>14</v>
+      </c>
+      <c r="D674">
+        <v>88</v>
+      </c>
+      <c r="E674" t="s">
+        <v>19</v>
+      </c>
+      <c r="F674" t="s">
+        <v>9</v>
+      </c>
+      <c r="G674">
+        <v>2019</v>
+      </c>
+      <c r="H674" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="675" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A675" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B675">
+        <v>8</v>
+      </c>
+      <c r="C675" t="s">
+        <v>14</v>
+      </c>
+      <c r="D675">
+        <v>111</v>
+      </c>
+      <c r="E675" t="s">
+        <v>19</v>
+      </c>
+      <c r="F675" t="s">
+        <v>9</v>
+      </c>
+      <c r="G675">
+        <v>2019</v>
+      </c>
+      <c r="H675" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="676" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A676" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B676">
+        <v>10</v>
+      </c>
+      <c r="C676" t="s">
+        <v>11</v>
+      </c>
+      <c r="D676">
+        <v>20</v>
+      </c>
+      <c r="E676" t="s">
+        <v>19</v>
+      </c>
+      <c r="F676" t="s">
+        <v>9</v>
+      </c>
+      <c r="G676">
+        <v>2019</v>
+      </c>
+      <c r="H676" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="677" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A677" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B677">
+        <v>30</v>
+      </c>
+      <c r="C677" t="s">
+        <v>11</v>
+      </c>
+      <c r="D677">
+        <v>30</v>
+      </c>
+      <c r="E677" t="s">
+        <v>19</v>
+      </c>
+      <c r="F677" t="s">
+        <v>9</v>
+      </c>
+      <c r="G677">
+        <v>2019</v>
+      </c>
+      <c r="H677" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="678" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A678" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B678">
+        <v>60</v>
+      </c>
+      <c r="C678" t="s">
+        <v>11</v>
+      </c>
+      <c r="D678">
+        <v>37</v>
+      </c>
+      <c r="E678" t="s">
+        <v>19</v>
+      </c>
+      <c r="F678" t="s">
+        <v>9</v>
+      </c>
+      <c r="G678">
+        <v>2019</v>
+      </c>
+      <c r="H678" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="679" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A679" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B679">
+        <v>4</v>
+      </c>
+      <c r="C679" t="s">
+        <v>8</v>
+      </c>
+      <c r="D679">
+        <v>51</v>
+      </c>
+      <c r="E679" t="s">
+        <v>19</v>
+      </c>
+      <c r="F679" t="s">
+        <v>9</v>
+      </c>
+      <c r="G679">
+        <v>2019</v>
+      </c>
+      <c r="H679" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="680" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A680" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B680">
+        <v>12</v>
+      </c>
+      <c r="C680" t="s">
+        <v>8</v>
+      </c>
+      <c r="D680">
+        <v>61</v>
+      </c>
+      <c r="E680" t="s">
+        <v>19</v>
+      </c>
+      <c r="F680" t="s">
+        <v>9</v>
+      </c>
+      <c r="G680">
+        <v>2019</v>
+      </c>
+      <c r="H680" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="681" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A681" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B681">
+        <v>24</v>
+      </c>
+      <c r="C681" t="s">
+        <v>8</v>
+      </c>
+      <c r="D681">
+        <v>71</v>
+      </c>
+      <c r="E681" t="s">
+        <v>19</v>
+      </c>
+      <c r="F681" t="s">
+        <v>9</v>
+      </c>
+      <c r="G681">
+        <v>2019</v>
+      </c>
+      <c r="H681" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="682" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A682" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B682">
+        <v>4</v>
+      </c>
+      <c r="C682" t="s">
+        <v>14</v>
+      </c>
+      <c r="D682">
+        <v>99</v>
+      </c>
+      <c r="E682" t="s">
+        <v>19</v>
+      </c>
+      <c r="F682" t="s">
+        <v>9</v>
+      </c>
+      <c r="G682">
+        <v>2019</v>
+      </c>
+      <c r="H682" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="683" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A683" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B683">
+        <v>8</v>
+      </c>
+      <c r="C683" t="s">
+        <v>14</v>
+      </c>
+      <c r="D683">
+        <v>123</v>
+      </c>
+      <c r="E683" t="s">
+        <v>19</v>
+      </c>
+      <c r="F683" t="s">
+        <v>9</v>
+      </c>
+      <c r="G683">
+        <v>2019</v>
+      </c>
+      <c r="H683" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="684" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A684" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B684">
+        <v>10</v>
+      </c>
+      <c r="C684" t="s">
+        <v>11</v>
+      </c>
+      <c r="D684">
+        <v>23</v>
+      </c>
+      <c r="E684" t="s">
+        <v>19</v>
+      </c>
+      <c r="F684" t="s">
+        <v>9</v>
+      </c>
+      <c r="G684">
+        <v>2019</v>
+      </c>
+      <c r="H684" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="685" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A685" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B685">
+        <v>30</v>
+      </c>
+      <c r="C685" t="s">
+        <v>11</v>
+      </c>
+      <c r="D685">
+        <v>36</v>
+      </c>
+      <c r="E685" t="s">
+        <v>19</v>
+      </c>
+      <c r="F685" t="s">
+        <v>9</v>
+      </c>
+      <c r="G685">
+        <v>2019</v>
+      </c>
+      <c r="H685" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="686" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A686" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B686">
+        <v>60</v>
+      </c>
+      <c r="C686" t="s">
+        <v>11</v>
+      </c>
+      <c r="D686">
+        <v>44</v>
+      </c>
+      <c r="E686" t="s">
+        <v>19</v>
+      </c>
+      <c r="F686" t="s">
+        <v>9</v>
+      </c>
+      <c r="G686">
+        <v>2019</v>
+      </c>
+      <c r="H686" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="687" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A687" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B687">
+        <v>4</v>
+      </c>
+      <c r="C687" t="s">
+        <v>8</v>
+      </c>
+      <c r="D687">
+        <v>60</v>
+      </c>
+      <c r="E687" t="s">
+        <v>19</v>
+      </c>
+      <c r="F687" t="s">
+        <v>9</v>
+      </c>
+      <c r="G687">
+        <v>2019</v>
+      </c>
+      <c r="H687" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="688" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A688" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B688">
+        <v>12</v>
+      </c>
+      <c r="C688" t="s">
+        <v>8</v>
+      </c>
+      <c r="D688">
+        <v>71</v>
+      </c>
+      <c r="E688" t="s">
+        <v>19</v>
+      </c>
+      <c r="F688" t="s">
+        <v>9</v>
+      </c>
+      <c r="G688">
+        <v>2019</v>
+      </c>
+      <c r="H688" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="689" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A689" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B689">
+        <v>24</v>
+      </c>
+      <c r="C689" t="s">
+        <v>8</v>
+      </c>
+      <c r="D689">
+        <v>81</v>
+      </c>
+      <c r="E689" t="s">
+        <v>19</v>
+      </c>
+      <c r="F689" t="s">
+        <v>9</v>
+      </c>
+      <c r="G689">
+        <v>2019</v>
+      </c>
+      <c r="H689" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="690" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A690" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B690">
+        <v>4</v>
+      </c>
+      <c r="C690" t="s">
+        <v>14</v>
+      </c>
+      <c r="D690">
+        <v>108</v>
+      </c>
+      <c r="E690" t="s">
+        <v>19</v>
+      </c>
+      <c r="F690" t="s">
+        <v>9</v>
+      </c>
+      <c r="G690">
+        <v>2019</v>
+      </c>
+      <c r="H690" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="691" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A691" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B691">
+        <v>8</v>
+      </c>
+      <c r="C691" t="s">
+        <v>14</v>
+      </c>
+      <c r="D691">
+        <v>132</v>
+      </c>
+      <c r="E691" t="s">
+        <v>19</v>
+      </c>
+      <c r="F691" t="s">
+        <v>9</v>
+      </c>
+      <c r="G691">
+        <v>2019</v>
+      </c>
+      <c r="H691" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="692" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A692" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B692">
+        <v>10</v>
+      </c>
+      <c r="C692" t="s">
+        <v>11</v>
+      </c>
+      <c r="D692">
+        <v>26</v>
+      </c>
+      <c r="E692" t="s">
+        <v>19</v>
+      </c>
+      <c r="F692" t="s">
+        <v>9</v>
+      </c>
+      <c r="G692">
+        <v>2019</v>
+      </c>
+      <c r="H692" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="693" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A693" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B693">
+        <v>30</v>
+      </c>
+      <c r="C693" t="s">
+        <v>11</v>
+      </c>
+      <c r="D693">
+        <v>42</v>
+      </c>
+      <c r="E693" t="s">
+        <v>19</v>
+      </c>
+      <c r="F693" t="s">
+        <v>9</v>
+      </c>
+      <c r="G693">
+        <v>2019</v>
+      </c>
+      <c r="H693" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="694" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A694" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B694">
+        <v>60</v>
+      </c>
+      <c r="C694" t="s">
+        <v>11</v>
+      </c>
+      <c r="D694">
+        <v>53</v>
+      </c>
+      <c r="E694" t="s">
+        <v>19</v>
+      </c>
+      <c r="F694" t="s">
+        <v>9</v>
+      </c>
+      <c r="G694">
+        <v>2019</v>
+      </c>
+      <c r="H694" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="695" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A695" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B695">
+        <v>4</v>
+      </c>
+      <c r="C695" t="s">
+        <v>8</v>
+      </c>
+      <c r="D695">
+        <v>71</v>
+      </c>
+      <c r="E695" t="s">
+        <v>19</v>
+      </c>
+      <c r="F695" t="s">
+        <v>9</v>
+      </c>
+      <c r="G695">
+        <v>2019</v>
+      </c>
+      <c r="H695" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="696" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A696" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B696">
+        <v>12</v>
+      </c>
+      <c r="C696" t="s">
+        <v>8</v>
+      </c>
+      <c r="D696">
+        <v>82</v>
+      </c>
+      <c r="E696" t="s">
+        <v>19</v>
+      </c>
+      <c r="F696" t="s">
+        <v>9</v>
+      </c>
+      <c r="G696">
+        <v>2019</v>
+      </c>
+      <c r="H696" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="697" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A697" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B697">
+        <v>24</v>
+      </c>
+      <c r="C697" t="s">
+        <v>8</v>
+      </c>
+      <c r="D697">
+        <v>90</v>
+      </c>
+      <c r="E697" t="s">
+        <v>19</v>
+      </c>
+      <c r="F697" t="s">
+        <v>9</v>
+      </c>
+      <c r="G697">
+        <v>2019</v>
+      </c>
+      <c r="H697" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="698" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A698" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B698">
+        <v>4</v>
+      </c>
+      <c r="C698" t="s">
+        <v>14</v>
+      </c>
+      <c r="D698">
+        <v>117</v>
+      </c>
+      <c r="E698" t="s">
+        <v>19</v>
+      </c>
+      <c r="F698" t="s">
+        <v>9</v>
+      </c>
+      <c r="G698">
+        <v>2019</v>
+      </c>
+      <c r="H698" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="699" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A699" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B699">
+        <v>8</v>
+      </c>
+      <c r="C699" t="s">
+        <v>14</v>
+      </c>
+      <c r="D699">
+        <v>139</v>
+      </c>
+      <c r="E699" t="s">
+        <v>19</v>
+      </c>
+      <c r="F699" t="s">
+        <v>9</v>
+      </c>
+      <c r="G699">
+        <v>2019</v>
+      </c>
+      <c r="H699" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="700" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A700" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B700">
+        <v>10</v>
+      </c>
+      <c r="C700" t="s">
+        <v>11</v>
+      </c>
+      <c r="D700">
+        <v>31</v>
+      </c>
+      <c r="E700" t="s">
+        <v>19</v>
+      </c>
+      <c r="F700" t="s">
+        <v>9</v>
+      </c>
+      <c r="G700">
+        <v>2019</v>
+      </c>
+      <c r="H700" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="701" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A701" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B701">
+        <v>30</v>
+      </c>
+      <c r="C701" t="s">
+        <v>11</v>
+      </c>
+      <c r="D701">
+        <v>51</v>
+      </c>
+      <c r="E701" t="s">
+        <v>19</v>
+      </c>
+      <c r="F701" t="s">
+        <v>9</v>
+      </c>
+      <c r="G701">
+        <v>2019</v>
+      </c>
+      <c r="H701" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="702" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A702" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B702">
+        <v>60</v>
+      </c>
+      <c r="C702" t="s">
+        <v>11</v>
+      </c>
+      <c r="D702">
+        <v>66</v>
+      </c>
+      <c r="E702" t="s">
+        <v>19</v>
+      </c>
+      <c r="F702" t="s">
+        <v>9</v>
+      </c>
+      <c r="G702">
+        <v>2019</v>
+      </c>
+      <c r="H702" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="703" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A703" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B703">
+        <v>4</v>
+      </c>
+      <c r="C703" t="s">
+        <v>8</v>
+      </c>
+      <c r="D703">
+        <v>83</v>
+      </c>
+      <c r="E703" t="s">
+        <v>19</v>
+      </c>
+      <c r="F703" t="s">
+        <v>9</v>
+      </c>
+      <c r="G703">
+        <v>2019</v>
+      </c>
+      <c r="H703" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="704" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A704" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B704">
+        <v>12</v>
+      </c>
+      <c r="C704" t="s">
+        <v>8</v>
+      </c>
+      <c r="D704">
+        <v>91</v>
+      </c>
+      <c r="E704" t="s">
+        <v>19</v>
+      </c>
+      <c r="F704" t="s">
+        <v>9</v>
+      </c>
+      <c r="G704">
+        <v>2019</v>
+      </c>
+      <c r="H704" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="705" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A705" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B705">
+        <v>24</v>
+      </c>
+      <c r="C705" t="s">
+        <v>8</v>
+      </c>
+      <c r="D705">
+        <v>103</v>
+      </c>
+      <c r="E705" t="s">
+        <v>19</v>
+      </c>
+      <c r="F705" t="s">
+        <v>9</v>
+      </c>
+      <c r="G705">
+        <v>2019</v>
+      </c>
+      <c r="H705" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="706" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A706" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B706">
+        <v>4</v>
+      </c>
+      <c r="C706" t="s">
+        <v>14</v>
+      </c>
+      <c r="D706">
+        <v>127</v>
+      </c>
+      <c r="E706" t="s">
+        <v>19</v>
+      </c>
+      <c r="F706" t="s">
+        <v>9</v>
+      </c>
+      <c r="G706">
+        <v>2019</v>
+      </c>
+      <c r="H706" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="707" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A707" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B707">
+        <v>8</v>
+      </c>
+      <c r="C707" t="s">
+        <v>14</v>
+      </c>
+      <c r="D707">
+        <v>147</v>
+      </c>
+      <c r="E707" t="s">
+        <v>19</v>
+      </c>
+      <c r="F707" t="s">
+        <v>9</v>
+      </c>
+      <c r="G707">
+        <v>2019</v>
+      </c>
+      <c r="H707" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="708" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A708" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B708">
+        <v>10</v>
+      </c>
+      <c r="C708" t="s">
+        <v>11</v>
+      </c>
+      <c r="D708">
+        <v>35</v>
+      </c>
+      <c r="E708" t="s">
+        <v>19</v>
+      </c>
+      <c r="F708" t="s">
+        <v>9</v>
+      </c>
+      <c r="G708">
+        <v>2019</v>
+      </c>
+      <c r="H708" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="709" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A709" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B709">
+        <v>30</v>
+      </c>
+      <c r="C709" t="s">
+        <v>11</v>
+      </c>
+      <c r="D709">
+        <v>61</v>
+      </c>
+      <c r="E709" t="s">
+        <v>19</v>
+      </c>
+      <c r="F709" t="s">
+        <v>9</v>
+      </c>
+      <c r="G709">
+        <v>2019</v>
+      </c>
+      <c r="H709" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="710" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A710" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B710">
+        <v>60</v>
+      </c>
+      <c r="C710" t="s">
+        <v>11</v>
+      </c>
+      <c r="D710">
+        <v>78</v>
+      </c>
+      <c r="E710" t="s">
+        <v>19</v>
+      </c>
+      <c r="F710" t="s">
+        <v>9</v>
+      </c>
+      <c r="G710">
+        <v>2019</v>
+      </c>
+      <c r="H710" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="711" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A711" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B711">
+        <v>4</v>
+      </c>
+      <c r="C711" t="s">
+        <v>8</v>
+      </c>
+      <c r="D711">
+        <v>96</v>
+      </c>
+      <c r="E711" t="s">
+        <v>19</v>
+      </c>
+      <c r="F711" t="s">
+        <v>9</v>
+      </c>
+      <c r="G711">
+        <v>2019</v>
+      </c>
+      <c r="H711" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="712" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A712" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B712">
+        <v>12</v>
+      </c>
+      <c r="C712" t="s">
+        <v>8</v>
+      </c>
+      <c r="D712">
+        <v>103</v>
+      </c>
+      <c r="E712" t="s">
+        <v>19</v>
+      </c>
+      <c r="F712" t="s">
+        <v>9</v>
+      </c>
+      <c r="G712">
+        <v>2019</v>
+      </c>
+      <c r="H712" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="713" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A713" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B713">
+        <v>24</v>
+      </c>
+      <c r="C713" t="s">
+        <v>8</v>
+      </c>
+      <c r="D713">
+        <v>113</v>
+      </c>
+      <c r="E713" t="s">
+        <v>19</v>
+      </c>
+      <c r="F713" t="s">
+        <v>9</v>
+      </c>
+      <c r="G713">
+        <v>2019</v>
+      </c>
+      <c r="H713" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="714" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A714" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B714">
+        <v>4</v>
+      </c>
+      <c r="C714" t="s">
+        <v>14</v>
+      </c>
+      <c r="D714">
+        <v>135</v>
+      </c>
+      <c r="E714" t="s">
+        <v>19</v>
+      </c>
+      <c r="F714" t="s">
+        <v>9</v>
+      </c>
+      <c r="G714">
+        <v>2019</v>
+      </c>
+      <c r="H714" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="715" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A715" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B715">
+        <v>8</v>
+      </c>
+      <c r="C715" t="s">
+        <v>14</v>
+      </c>
+      <c r="D715">
+        <v>153</v>
+      </c>
+      <c r="E715" t="s">
+        <v>19</v>
+      </c>
+      <c r="F715" t="s">
+        <v>9</v>
+      </c>
+      <c r="G715">
+        <v>2019</v>
+      </c>
+      <c r="H715" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="716" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A716" s="4">
+        <f>0.001</f>
+        <v>1E-3</v>
+      </c>
+      <c r="B716">
+        <v>10</v>
+      </c>
+      <c r="C716" t="s">
+        <v>11</v>
+      </c>
+      <c r="D716">
+        <v>40</v>
+      </c>
+      <c r="E716" t="s">
+        <v>19</v>
+      </c>
+      <c r="F716" t="s">
+        <v>9</v>
+      </c>
+      <c r="G716">
+        <v>2019</v>
+      </c>
+      <c r="H716" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="717" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A717" s="4">
+        <f t="shared" ref="A717:A723" si="4">0.001</f>
+        <v>1E-3</v>
+      </c>
+      <c r="B717">
+        <v>30</v>
+      </c>
+      <c r="C717" t="s">
+        <v>11</v>
+      </c>
+      <c r="D717">
+        <v>71</v>
+      </c>
+      <c r="E717" t="s">
+        <v>19</v>
+      </c>
+      <c r="F717" t="s">
+        <v>9</v>
+      </c>
+      <c r="G717">
+        <v>2019</v>
+      </c>
+      <c r="H717" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="718" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A718" s="4">
+        <f t="shared" si="4"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B718">
+        <v>60</v>
+      </c>
+      <c r="C718" t="s">
+        <v>11</v>
+      </c>
+      <c r="D718">
+        <v>93</v>
+      </c>
+      <c r="E718" t="s">
+        <v>19</v>
+      </c>
+      <c r="F718" t="s">
+        <v>9</v>
+      </c>
+      <c r="G718">
+        <v>2019</v>
+      </c>
+      <c r="H718" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="719" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A719" s="4">
+        <f t="shared" si="4"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B719">
+        <v>4</v>
+      </c>
+      <c r="C719" t="s">
+        <v>8</v>
+      </c>
+      <c r="D719">
+        <v>113</v>
+      </c>
+      <c r="E719" t="s">
+        <v>19</v>
+      </c>
+      <c r="F719" t="s">
+        <v>9</v>
+      </c>
+      <c r="G719">
+        <v>2019</v>
+      </c>
+      <c r="H719" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="720" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A720" s="4">
+        <f t="shared" si="4"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B720">
+        <v>12</v>
+      </c>
+      <c r="C720" t="s">
+        <v>8</v>
+      </c>
+      <c r="D720">
+        <v>117</v>
+      </c>
+      <c r="E720" t="s">
+        <v>19</v>
+      </c>
+      <c r="F720" t="s">
+        <v>9</v>
+      </c>
+      <c r="G720">
+        <v>2019</v>
+      </c>
+      <c r="H720" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="721" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A721" s="4">
+        <f t="shared" si="4"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B721">
+        <v>24</v>
+      </c>
+      <c r="C721" t="s">
+        <v>8</v>
+      </c>
+      <c r="D721">
+        <v>124</v>
+      </c>
+      <c r="E721" t="s">
+        <v>19</v>
+      </c>
+      <c r="F721" t="s">
+        <v>9</v>
+      </c>
+      <c r="G721">
+        <v>2019</v>
+      </c>
+      <c r="H721" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="722" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A722" s="4">
+        <f t="shared" si="4"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B722">
+        <v>4</v>
+      </c>
+      <c r="C722" t="s">
+        <v>14</v>
+      </c>
+      <c r="D722">
+        <v>142</v>
+      </c>
+      <c r="E722" t="s">
+        <v>19</v>
+      </c>
+      <c r="F722" t="s">
+        <v>9</v>
+      </c>
+      <c r="G722">
+        <v>2019</v>
+      </c>
+      <c r="H722" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="723" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A723" s="4">
+        <f t="shared" si="4"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B723">
+        <v>8</v>
+      </c>
+      <c r="C723" t="s">
+        <v>14</v>
+      </c>
+      <c r="D723">
+        <v>157</v>
+      </c>
+      <c r="E723" t="s">
+        <v>19</v>
+      </c>
+      <c r="F723" t="s">
+        <v>9</v>
+      </c>
+      <c r="G723">
+        <v>2019</v>
+      </c>
+      <c r="H723" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="724" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A724" s="1">
+        <v>2</v>
+      </c>
+      <c r="B724">
+        <v>10</v>
+      </c>
+      <c r="C724" t="s">
+        <v>11</v>
+      </c>
+      <c r="D724">
+        <v>8</v>
+      </c>
+      <c r="E724" t="s">
+        <v>19</v>
+      </c>
+      <c r="F724" t="s">
+        <v>9</v>
+      </c>
+      <c r="G724">
+        <v>2019</v>
+      </c>
+      <c r="H724" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="725" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A725" s="1">
+        <v>2</v>
+      </c>
+      <c r="B725">
+        <v>30</v>
+      </c>
+      <c r="C725" t="s">
+        <v>11</v>
+      </c>
+      <c r="D725">
+        <v>10</v>
+      </c>
+      <c r="E725" t="s">
+        <v>19</v>
+      </c>
+      <c r="F725" t="s">
+        <v>9</v>
+      </c>
+      <c r="G725">
+        <v>2019</v>
+      </c>
+      <c r="H725" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="726" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A726" s="1">
+        <v>2</v>
+      </c>
+      <c r="B726">
+        <v>60</v>
+      </c>
+      <c r="C726" t="s">
+        <v>11</v>
+      </c>
+      <c r="D726">
+        <v>13</v>
+      </c>
+      <c r="E726" t="s">
+        <v>19</v>
+      </c>
+      <c r="F726" t="s">
+        <v>9</v>
+      </c>
+      <c r="G726">
+        <v>2019</v>
+      </c>
+      <c r="H726" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="727" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A727" s="1">
+        <v>2</v>
+      </c>
+      <c r="B727">
+        <v>4</v>
+      </c>
+      <c r="C727" t="s">
+        <v>8</v>
+      </c>
+      <c r="D727">
+        <v>19</v>
+      </c>
+      <c r="E727" t="s">
+        <v>19</v>
+      </c>
+      <c r="F727" t="s">
+        <v>9</v>
+      </c>
+      <c r="G727">
+        <v>2019</v>
+      </c>
+      <c r="H727" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="728" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A728" s="1">
+        <v>2</v>
+      </c>
+      <c r="B728">
+        <v>12</v>
+      </c>
+      <c r="C728" t="s">
+        <v>8</v>
+      </c>
+      <c r="D728">
+        <v>25</v>
+      </c>
+      <c r="E728" t="s">
+        <v>19</v>
+      </c>
+      <c r="F728" t="s">
+        <v>9</v>
+      </c>
+      <c r="G728">
+        <v>2019</v>
+      </c>
+      <c r="H728" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="729" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A729" s="1">
+        <v>2</v>
+      </c>
+      <c r="B729">
+        <v>24</v>
+      </c>
+      <c r="C729" t="s">
+        <v>8</v>
+      </c>
+      <c r="D729">
+        <v>30</v>
+      </c>
+      <c r="E729" t="s">
+        <v>19</v>
+      </c>
+      <c r="F729" t="s">
+        <v>9</v>
+      </c>
+      <c r="G729">
+        <v>2019</v>
+      </c>
+      <c r="H729" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="730" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A730" s="1">
+        <v>2</v>
+      </c>
+      <c r="B730">
+        <v>4</v>
+      </c>
+      <c r="C730" t="s">
+        <v>14</v>
+      </c>
+      <c r="D730">
+        <v>50</v>
+      </c>
+      <c r="E730" t="s">
+        <v>19</v>
+      </c>
+      <c r="F730" t="s">
+        <v>9</v>
+      </c>
+      <c r="G730">
+        <v>2019</v>
+      </c>
+      <c r="H730" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="731" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A731" s="1">
+        <v>2</v>
+      </c>
+      <c r="B731">
+        <v>8</v>
+      </c>
+      <c r="C731" t="s">
+        <v>14</v>
+      </c>
+      <c r="D731">
+        <v>68</v>
+      </c>
+      <c r="E731" t="s">
+        <v>19</v>
+      </c>
+      <c r="F731" t="s">
+        <v>9</v>
+      </c>
+      <c r="G731">
+        <v>2019</v>
+      </c>
+      <c r="H731" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="732" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A732" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B732">
+        <v>10</v>
+      </c>
+      <c r="C732" t="s">
+        <v>11</v>
+      </c>
+      <c r="D732">
+        <v>12</v>
+      </c>
+      <c r="E732" t="s">
+        <v>19</v>
+      </c>
+      <c r="F732" t="s">
+        <v>9</v>
+      </c>
+      <c r="G732">
+        <v>2019</v>
+      </c>
+      <c r="H732" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="733" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A733" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B733">
+        <v>30</v>
+      </c>
+      <c r="C733" t="s">
+        <v>11</v>
+      </c>
+      <c r="D733">
+        <v>17</v>
+      </c>
+      <c r="E733" t="s">
+        <v>19</v>
+      </c>
+      <c r="F733" t="s">
+        <v>9</v>
+      </c>
+      <c r="G733">
+        <v>2019</v>
+      </c>
+      <c r="H733" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="734" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A734" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B734">
+        <v>60</v>
+      </c>
+      <c r="C734" t="s">
+        <v>11</v>
+      </c>
+      <c r="D734">
+        <v>20</v>
+      </c>
+      <c r="E734" t="s">
+        <v>19</v>
+      </c>
+      <c r="F734" t="s">
+        <v>9</v>
+      </c>
+      <c r="G734">
+        <v>2019</v>
+      </c>
+      <c r="H734" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="735" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A735" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B735">
+        <v>4</v>
+      </c>
+      <c r="C735" t="s">
+        <v>8</v>
+      </c>
+      <c r="D735">
+        <v>28</v>
+      </c>
+      <c r="E735" t="s">
+        <v>19</v>
+      </c>
+      <c r="F735" t="s">
+        <v>9</v>
+      </c>
+      <c r="G735">
+        <v>2019</v>
+      </c>
+      <c r="H735" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="736" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A736" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B736">
+        <v>12</v>
+      </c>
+      <c r="C736" t="s">
+        <v>8</v>
+      </c>
+      <c r="D736">
+        <v>37</v>
+      </c>
+      <c r="E736" t="s">
+        <v>19</v>
+      </c>
+      <c r="F736" t="s">
+        <v>9</v>
+      </c>
+      <c r="G736">
+        <v>2019</v>
+      </c>
+      <c r="H736" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="737" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A737" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B737">
+        <v>24</v>
+      </c>
+      <c r="C737" t="s">
+        <v>8</v>
+      </c>
+      <c r="D737">
+        <v>44</v>
+      </c>
+      <c r="E737" t="s">
+        <v>19</v>
+      </c>
+      <c r="F737" t="s">
+        <v>9</v>
+      </c>
+      <c r="G737">
+        <v>2019</v>
+      </c>
+      <c r="H737" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="738" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A738" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B738">
+        <v>4</v>
+      </c>
+      <c r="C738" t="s">
+        <v>14</v>
+      </c>
+      <c r="D738">
+        <v>69</v>
+      </c>
+      <c r="E738" t="s">
+        <v>19</v>
+      </c>
+      <c r="F738" t="s">
+        <v>9</v>
+      </c>
+      <c r="G738">
+        <v>2019</v>
+      </c>
+      <c r="H738" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="739" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A739" s="2">
+        <v>0.5</v>
+      </c>
+      <c r="B739">
+        <v>8</v>
+      </c>
+      <c r="C739" t="s">
+        <v>14</v>
+      </c>
+      <c r="D739">
+        <v>91</v>
+      </c>
+      <c r="E739" t="s">
+        <v>19</v>
+      </c>
+      <c r="F739" t="s">
+        <v>9</v>
+      </c>
+      <c r="G739">
+        <v>2019</v>
+      </c>
+      <c r="H739" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="740" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A740" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B740">
+        <v>10</v>
+      </c>
+      <c r="C740" t="s">
+        <v>11</v>
+      </c>
+      <c r="D740">
+        <v>18</v>
+      </c>
+      <c r="E740" t="s">
+        <v>19</v>
+      </c>
+      <c r="F740" t="s">
+        <v>9</v>
+      </c>
+      <c r="G740">
+        <v>2019</v>
+      </c>
+      <c r="H740" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="741" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A741" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B741">
+        <v>30</v>
+      </c>
+      <c r="C741" t="s">
+        <v>11</v>
+      </c>
+      <c r="D741">
+        <v>27</v>
+      </c>
+      <c r="E741" t="s">
+        <v>19</v>
+      </c>
+      <c r="F741" t="s">
+        <v>9</v>
+      </c>
+      <c r="G741">
+        <v>2019</v>
+      </c>
+      <c r="H741" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="742" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A742" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B742">
+        <v>60</v>
+      </c>
+      <c r="C742" t="s">
+        <v>11</v>
+      </c>
+      <c r="D742">
+        <v>33</v>
+      </c>
+      <c r="E742" t="s">
+        <v>19</v>
+      </c>
+      <c r="F742" t="s">
+        <v>9</v>
+      </c>
+      <c r="G742">
+        <v>2019</v>
+      </c>
+      <c r="H742" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="743" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A743" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B743">
+        <v>4</v>
+      </c>
+      <c r="C743" t="s">
+        <v>8</v>
+      </c>
+      <c r="D743">
+        <v>45</v>
+      </c>
+      <c r="E743" t="s">
+        <v>19</v>
+      </c>
+      <c r="F743" t="s">
+        <v>9</v>
+      </c>
+      <c r="G743">
+        <v>2019</v>
+      </c>
+      <c r="H743" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="744" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A744" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B744">
+        <v>12</v>
+      </c>
+      <c r="C744" t="s">
+        <v>8</v>
+      </c>
+      <c r="D744">
+        <v>56</v>
+      </c>
+      <c r="E744" t="s">
+        <v>19</v>
+      </c>
+      <c r="F744" t="s">
+        <v>9</v>
+      </c>
+      <c r="G744">
+        <v>2019</v>
+      </c>
+      <c r="H744" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="745" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A745" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B745">
+        <v>24</v>
+      </c>
+      <c r="C745" t="s">
+        <v>8</v>
+      </c>
+      <c r="D745">
+        <v>66</v>
+      </c>
+      <c r="E745" t="s">
+        <v>19</v>
+      </c>
+      <c r="F745" t="s">
+        <v>9</v>
+      </c>
+      <c r="G745">
+        <v>2019</v>
+      </c>
+      <c r="H745" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="746" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A746" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B746">
+        <v>4</v>
+      </c>
+      <c r="C746" t="s">
+        <v>14</v>
+      </c>
+      <c r="D746">
+        <v>96</v>
+      </c>
+      <c r="E746" t="s">
+        <v>19</v>
+      </c>
+      <c r="F746" t="s">
+        <v>9</v>
+      </c>
+      <c r="G746">
+        <v>2019</v>
+      </c>
+      <c r="H746" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="747" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A747" s="2">
+        <v>0.1</v>
+      </c>
+      <c r="B747">
+        <v>8</v>
+      </c>
+      <c r="C747" t="s">
+        <v>14</v>
+      </c>
+      <c r="D747">
+        <v>122</v>
+      </c>
+      <c r="E747" t="s">
+        <v>19</v>
+      </c>
+      <c r="F747" t="s">
+        <v>9</v>
+      </c>
+      <c r="G747">
+        <v>2019</v>
+      </c>
+      <c r="H747" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="748" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A748" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B748">
+        <v>10</v>
+      </c>
+      <c r="C748" t="s">
+        <v>11</v>
+      </c>
+      <c r="D748">
+        <v>23</v>
+      </c>
+      <c r="E748" t="s">
+        <v>19</v>
+      </c>
+      <c r="F748" t="s">
+        <v>9</v>
+      </c>
+      <c r="G748">
+        <v>2019</v>
+      </c>
+      <c r="H748" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="749" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A749" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B749">
+        <v>30</v>
+      </c>
+      <c r="C749" t="s">
+        <v>11</v>
+      </c>
+      <c r="D749">
+        <v>35</v>
+      </c>
+      <c r="E749" t="s">
+        <v>19</v>
+      </c>
+      <c r="F749" t="s">
+        <v>9</v>
+      </c>
+      <c r="G749">
+        <v>2019</v>
+      </c>
+      <c r="H749" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="750" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A750" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B750">
+        <v>60</v>
+      </c>
+      <c r="C750" t="s">
+        <v>11</v>
+      </c>
+      <c r="D750">
+        <v>43</v>
+      </c>
+      <c r="E750" t="s">
+        <v>19</v>
+      </c>
+      <c r="F750" t="s">
+        <v>9</v>
+      </c>
+      <c r="G750">
+        <v>2019</v>
+      </c>
+      <c r="H750" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="751" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A751" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B751">
+        <v>4</v>
+      </c>
+      <c r="C751" t="s">
+        <v>8</v>
+      </c>
+      <c r="D751">
+        <v>59</v>
+      </c>
+      <c r="E751" t="s">
+        <v>19</v>
+      </c>
+      <c r="F751" t="s">
+        <v>9</v>
+      </c>
+      <c r="G751">
+        <v>2019</v>
+      </c>
+      <c r="H751" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="752" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A752" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B752">
+        <v>12</v>
+      </c>
+      <c r="C752" t="s">
+        <v>8</v>
+      </c>
+      <c r="D752">
+        <v>71</v>
+      </c>
+      <c r="E752" t="s">
+        <v>19</v>
+      </c>
+      <c r="F752" t="s">
+        <v>9</v>
+      </c>
+      <c r="G752">
+        <v>2019</v>
+      </c>
+      <c r="H752" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="753" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A753" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B753">
+        <v>24</v>
+      </c>
+      <c r="C753" t="s">
+        <v>8</v>
+      </c>
+      <c r="D753">
+        <v>83</v>
+      </c>
+      <c r="E753" t="s">
+        <v>19</v>
+      </c>
+      <c r="F753" t="s">
+        <v>9</v>
+      </c>
+      <c r="G753">
+        <v>2019</v>
+      </c>
+      <c r="H753" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="754" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A754" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B754">
+        <v>4</v>
+      </c>
+      <c r="C754" t="s">
+        <v>14</v>
+      </c>
+      <c r="D754">
+        <v>115</v>
+      </c>
+      <c r="E754" t="s">
+        <v>19</v>
+      </c>
+      <c r="F754" t="s">
+        <v>9</v>
+      </c>
+      <c r="G754">
+        <v>2019</v>
+      </c>
+      <c r="H754" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="755" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A755" s="3">
+        <v>0.04</v>
+      </c>
+      <c r="B755">
+        <v>8</v>
+      </c>
+      <c r="C755" t="s">
+        <v>14</v>
+      </c>
+      <c r="D755">
+        <v>142</v>
+      </c>
+      <c r="E755" t="s">
+        <v>19</v>
+      </c>
+      <c r="F755" t="s">
+        <v>9</v>
+      </c>
+      <c r="G755">
+        <v>2019</v>
+      </c>
+      <c r="H755" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="756" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A756" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B756">
+        <v>10</v>
+      </c>
+      <c r="C756" t="s">
+        <v>11</v>
+      </c>
+      <c r="D756">
+        <v>27</v>
+      </c>
+      <c r="E756" t="s">
+        <v>19</v>
+      </c>
+      <c r="F756" t="s">
+        <v>9</v>
+      </c>
+      <c r="G756">
+        <v>2019</v>
+      </c>
+      <c r="H756" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="757" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A757" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B757">
+        <v>30</v>
+      </c>
+      <c r="C757" t="s">
+        <v>11</v>
+      </c>
+      <c r="D757">
+        <v>42</v>
+      </c>
+      <c r="E757" t="s">
+        <v>19</v>
+      </c>
+      <c r="F757" t="s">
+        <v>9</v>
+      </c>
+      <c r="G757">
+        <v>2019</v>
+      </c>
+      <c r="H757" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="758" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A758" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B758">
+        <v>60</v>
+      </c>
+      <c r="C758" t="s">
+        <v>11</v>
+      </c>
+      <c r="D758">
+        <v>52</v>
+      </c>
+      <c r="E758" t="s">
+        <v>19</v>
+      </c>
+      <c r="F758" t="s">
+        <v>9</v>
+      </c>
+      <c r="G758">
+        <v>2019</v>
+      </c>
+      <c r="H758" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="759" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A759" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B759">
+        <v>4</v>
+      </c>
+      <c r="C759" t="s">
+        <v>8</v>
+      </c>
+      <c r="D759">
+        <v>71</v>
+      </c>
+      <c r="E759" t="s">
+        <v>19</v>
+      </c>
+      <c r="F759" t="s">
+        <v>9</v>
+      </c>
+      <c r="G759">
+        <v>2019</v>
+      </c>
+      <c r="H759" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="760" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A760" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B760">
+        <v>12</v>
+      </c>
+      <c r="C760" t="s">
+        <v>8</v>
+      </c>
+      <c r="D760">
+        <v>83</v>
+      </c>
+      <c r="E760" t="s">
+        <v>19</v>
+      </c>
+      <c r="F760" t="s">
+        <v>9</v>
+      </c>
+      <c r="G760">
+        <v>2019</v>
+      </c>
+      <c r="H760" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="761" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A761" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B761">
+        <v>24</v>
+      </c>
+      <c r="C761" t="s">
+        <v>8</v>
+      </c>
+      <c r="D761">
+        <v>95</v>
+      </c>
+      <c r="E761" t="s">
+        <v>19</v>
+      </c>
+      <c r="F761" t="s">
+        <v>9</v>
+      </c>
+      <c r="G761">
+        <v>2019</v>
+      </c>
+      <c r="H761" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="762" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A762" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B762">
+        <v>4</v>
+      </c>
+      <c r="C762" t="s">
+        <v>14</v>
+      </c>
+      <c r="D762">
+        <v>127</v>
+      </c>
+      <c r="E762" t="s">
+        <v>19</v>
+      </c>
+      <c r="F762" t="s">
+        <v>9</v>
+      </c>
+      <c r="G762">
+        <v>2019</v>
+      </c>
+      <c r="H762" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="763" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A763" s="3">
+        <v>0.02</v>
+      </c>
+      <c r="B763">
+        <v>8</v>
+      </c>
+      <c r="C763" t="s">
+        <v>14</v>
+      </c>
+      <c r="D763">
+        <v>154</v>
+      </c>
+      <c r="E763" t="s">
+        <v>19</v>
+      </c>
+      <c r="F763" t="s">
+        <v>9</v>
+      </c>
+      <c r="G763">
+        <v>2019</v>
+      </c>
+      <c r="H763" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="764" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A764" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B764">
+        <v>10</v>
+      </c>
+      <c r="C764" t="s">
+        <v>11</v>
+      </c>
+      <c r="D764">
+        <v>32</v>
+      </c>
+      <c r="E764" t="s">
+        <v>19</v>
+      </c>
+      <c r="F764" t="s">
+        <v>9</v>
+      </c>
+      <c r="G764">
+        <v>2019</v>
+      </c>
+      <c r="H764" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="765" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A765" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B765">
+        <v>30</v>
+      </c>
+      <c r="C765" t="s">
+        <v>11</v>
+      </c>
+      <c r="D765">
+        <v>51</v>
+      </c>
+      <c r="E765" t="s">
+        <v>19</v>
+      </c>
+      <c r="F765" t="s">
+        <v>9</v>
+      </c>
+      <c r="G765">
+        <v>2019</v>
+      </c>
+      <c r="H765" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="766" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A766" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B766">
+        <v>60</v>
+      </c>
+      <c r="C766" t="s">
+        <v>11</v>
+      </c>
+      <c r="D766">
+        <v>64</v>
+      </c>
+      <c r="E766" t="s">
+        <v>19</v>
+      </c>
+      <c r="F766" t="s">
+        <v>9</v>
+      </c>
+      <c r="G766">
+        <v>2019</v>
+      </c>
+      <c r="H766" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="767" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A767" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B767">
+        <v>4</v>
+      </c>
+      <c r="C767" t="s">
+        <v>8</v>
+      </c>
+      <c r="D767">
+        <v>87</v>
+      </c>
+      <c r="E767" t="s">
+        <v>19</v>
+      </c>
+      <c r="F767" t="s">
+        <v>9</v>
+      </c>
+      <c r="G767">
+        <v>2019</v>
+      </c>
+      <c r="H767" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="768" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A768" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B768">
+        <v>12</v>
+      </c>
+      <c r="C768" t="s">
+        <v>8</v>
+      </c>
+      <c r="D768">
+        <v>100</v>
+      </c>
+      <c r="E768" t="s">
+        <v>19</v>
+      </c>
+      <c r="F768" t="s">
+        <v>9</v>
+      </c>
+      <c r="G768">
+        <v>2019</v>
+      </c>
+      <c r="H768" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="769" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A769" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B769">
+        <v>24</v>
+      </c>
+      <c r="C769" t="s">
+        <v>8</v>
+      </c>
+      <c r="D769">
+        <v>110</v>
+      </c>
+      <c r="E769" t="s">
+        <v>19</v>
+      </c>
+      <c r="F769" t="s">
+        <v>9</v>
+      </c>
+      <c r="G769">
+        <v>2019</v>
+      </c>
+      <c r="H769" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="770" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A770" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B770">
+        <v>4</v>
+      </c>
+      <c r="C770" t="s">
+        <v>14</v>
+      </c>
+      <c r="D770">
+        <v>142</v>
+      </c>
+      <c r="E770" t="s">
+        <v>19</v>
+      </c>
+      <c r="F770" t="s">
+        <v>9</v>
+      </c>
+      <c r="G770">
+        <v>2019</v>
+      </c>
+      <c r="H770" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="771" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A771" s="3">
+        <v>0.01</v>
+      </c>
+      <c r="B771">
+        <v>8</v>
+      </c>
+      <c r="C771" t="s">
+        <v>14</v>
+      </c>
+      <c r="D771">
+        <v>169</v>
+      </c>
+      <c r="E771" t="s">
+        <v>19</v>
+      </c>
+      <c r="F771" t="s">
+        <v>9</v>
+      </c>
+      <c r="G771">
+        <v>2019</v>
+      </c>
+      <c r="H771" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="772" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A772" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B772">
+        <v>10</v>
+      </c>
+      <c r="C772" t="s">
+        <v>11</v>
+      </c>
+      <c r="D772">
+        <v>40</v>
+      </c>
+      <c r="E772" t="s">
+        <v>19</v>
+      </c>
+      <c r="F772" t="s">
+        <v>9</v>
+      </c>
+      <c r="G772">
+        <v>2019</v>
+      </c>
+      <c r="H772" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="773" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A773" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B773">
+        <v>30</v>
+      </c>
+      <c r="C773" t="s">
+        <v>11</v>
+      </c>
+      <c r="D773">
+        <v>66</v>
+      </c>
+      <c r="E773" t="s">
+        <v>19</v>
+      </c>
+      <c r="F773" t="s">
+        <v>9</v>
+      </c>
+      <c r="G773">
+        <v>2019</v>
+      </c>
+      <c r="H773" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="774" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A774" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B774">
+        <v>60</v>
+      </c>
+      <c r="C774" t="s">
+        <v>11</v>
+      </c>
+      <c r="D774">
+        <v>84</v>
+      </c>
+      <c r="E774" t="s">
+        <v>19</v>
+      </c>
+      <c r="F774" t="s">
+        <v>9</v>
+      </c>
+      <c r="G774">
+        <v>2019</v>
+      </c>
+      <c r="H774" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="775" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A775" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B775">
+        <v>4</v>
+      </c>
+      <c r="C775" t="s">
+        <v>8</v>
+      </c>
+      <c r="D775">
+        <v>106</v>
+      </c>
+      <c r="E775" t="s">
+        <v>19</v>
+      </c>
+      <c r="F775" t="s">
+        <v>9</v>
+      </c>
+      <c r="G775">
+        <v>2019</v>
+      </c>
+      <c r="H775" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="776" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A776" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B776">
+        <v>12</v>
+      </c>
+      <c r="C776" t="s">
+        <v>8</v>
+      </c>
+      <c r="D776">
+        <v>116</v>
+      </c>
+      <c r="E776" t="s">
+        <v>19</v>
+      </c>
+      <c r="F776" t="s">
+        <v>9</v>
+      </c>
+      <c r="G776">
+        <v>2019</v>
+      </c>
+      <c r="H776" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="777" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A777" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B777">
+        <v>24</v>
+      </c>
+      <c r="C777" t="s">
+        <v>8</v>
+      </c>
+      <c r="D777">
+        <v>132</v>
+      </c>
+      <c r="E777" t="s">
+        <v>19</v>
+      </c>
+      <c r="F777" t="s">
+        <v>9</v>
+      </c>
+      <c r="G777">
+        <v>2019</v>
+      </c>
+      <c r="H777" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="778" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A778" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B778">
+        <v>4</v>
+      </c>
+      <c r="C778" t="s">
+        <v>14</v>
+      </c>
+      <c r="D778">
+        <v>163</v>
+      </c>
+      <c r="E778" t="s">
+        <v>19</v>
+      </c>
+      <c r="F778" t="s">
+        <v>9</v>
+      </c>
+      <c r="G778">
+        <v>2019</v>
+      </c>
+      <c r="H778" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="779" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A779" s="4">
+        <v>4.0000000000000001E-3</v>
+      </c>
+      <c r="B779">
+        <v>8</v>
+      </c>
+      <c r="C779" t="s">
+        <v>14</v>
+      </c>
+      <c r="D779">
+        <v>188</v>
+      </c>
+      <c r="E779" t="s">
+        <v>19</v>
+      </c>
+      <c r="F779" t="s">
+        <v>9</v>
+      </c>
+      <c r="G779">
+        <v>2019</v>
+      </c>
+      <c r="H779" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="780" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A780" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B780">
+        <v>10</v>
+      </c>
+      <c r="C780" t="s">
+        <v>11</v>
+      </c>
+      <c r="D780">
+        <v>48</v>
+      </c>
+      <c r="E780" t="s">
+        <v>19</v>
+      </c>
+      <c r="F780" t="s">
+        <v>9</v>
+      </c>
+      <c r="G780">
+        <v>2019</v>
+      </c>
+      <c r="H780" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="781" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A781" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B781">
+        <v>30</v>
+      </c>
+      <c r="C781" t="s">
+        <v>11</v>
+      </c>
+      <c r="D781">
+        <v>82</v>
+      </c>
+      <c r="E781" t="s">
+        <v>19</v>
+      </c>
+      <c r="F781" t="s">
+        <v>9</v>
+      </c>
+      <c r="G781">
+        <v>2019</v>
+      </c>
+      <c r="H781" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="782" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A782" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B782">
+        <v>60</v>
+      </c>
+      <c r="C782" t="s">
+        <v>11</v>
+      </c>
+      <c r="D782">
+        <v>106</v>
+      </c>
+      <c r="E782" t="s">
+        <v>19</v>
+      </c>
+      <c r="F782" t="s">
+        <v>9</v>
+      </c>
+      <c r="G782">
+        <v>2019</v>
+      </c>
+      <c r="H782" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="783" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A783" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B783">
+        <v>4</v>
+      </c>
+      <c r="C783" t="s">
+        <v>8</v>
+      </c>
+      <c r="D783">
+        <v>131</v>
+      </c>
+      <c r="E783" t="s">
+        <v>19</v>
+      </c>
+      <c r="F783" t="s">
+        <v>9</v>
+      </c>
+      <c r="G783">
+        <v>2019</v>
+      </c>
+      <c r="H783" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="784" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A784" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B784">
+        <v>12</v>
+      </c>
+      <c r="C784" t="s">
+        <v>8</v>
+      </c>
+      <c r="D784">
+        <v>140</v>
+      </c>
+      <c r="E784" t="s">
+        <v>19</v>
+      </c>
+      <c r="F784" t="s">
+        <v>9</v>
+      </c>
+      <c r="G784">
+        <v>2019</v>
+      </c>
+      <c r="H784" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="785" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A785" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B785">
+        <v>24</v>
+      </c>
+      <c r="C785" t="s">
+        <v>8</v>
+      </c>
+      <c r="D785">
+        <v>154</v>
+      </c>
+      <c r="E785" t="s">
+        <v>19</v>
+      </c>
+      <c r="F785" t="s">
+        <v>9</v>
+      </c>
+      <c r="G785">
+        <v>2019</v>
+      </c>
+      <c r="H785" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="786" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A786" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B786">
+        <v>4</v>
+      </c>
+      <c r="C786" t="s">
+        <v>14</v>
+      </c>
+      <c r="D786">
+        <v>183</v>
+      </c>
+      <c r="E786" t="s">
+        <v>19</v>
+      </c>
+      <c r="F786" t="s">
+        <v>9</v>
+      </c>
+      <c r="G786">
+        <v>2019</v>
+      </c>
+      <c r="H786" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="787" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A787" s="4">
+        <v>2E-3</v>
+      </c>
+      <c r="B787">
+        <v>8</v>
+      </c>
+      <c r="C787" t="s">
+        <v>14</v>
+      </c>
+      <c r="D787">
+        <v>208</v>
+      </c>
+      <c r="E787" t="s">
+        <v>19</v>
+      </c>
+      <c r="F787" t="s">
+        <v>9</v>
+      </c>
+      <c r="G787">
+        <v>2019</v>
+      </c>
+      <c r="H787" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="788" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A788" s="4">
+        <f>0.001</f>
+        <v>1E-3</v>
+      </c>
+      <c r="B788">
+        <v>10</v>
+      </c>
+      <c r="C788" t="s">
+        <v>11</v>
+      </c>
+      <c r="D788">
+        <v>57</v>
+      </c>
+      <c r="E788" t="s">
+        <v>19</v>
+      </c>
+      <c r="F788" t="s">
+        <v>9</v>
+      </c>
+      <c r="G788">
+        <v>2019</v>
+      </c>
+      <c r="H788" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="789" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A789" s="4">
+        <f t="shared" ref="A789:A795" si="5">0.001</f>
+        <v>1E-3</v>
+      </c>
+      <c r="B789">
+        <v>30</v>
+      </c>
+      <c r="C789" t="s">
+        <v>11</v>
+      </c>
+      <c r="D789">
+        <v>102</v>
+      </c>
+      <c r="E789" t="s">
+        <v>19</v>
+      </c>
+      <c r="F789" t="s">
+        <v>9</v>
+      </c>
+      <c r="G789">
+        <v>2019</v>
+      </c>
+      <c r="H789" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="790" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A790" s="4">
+        <f t="shared" si="5"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B790">
+        <v>60</v>
+      </c>
+      <c r="C790" t="s">
+        <v>11</v>
+      </c>
+      <c r="D790">
+        <v>133</v>
+      </c>
+      <c r="E790" t="s">
+        <v>19</v>
+      </c>
+      <c r="F790" t="s">
+        <v>9</v>
+      </c>
+      <c r="G790">
+        <v>2019</v>
+      </c>
+      <c r="H790" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="791" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A791" s="4">
+        <f t="shared" si="5"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B791">
+        <v>4</v>
+      </c>
+      <c r="C791" t="s">
+        <v>8</v>
+      </c>
+      <c r="D791">
+        <v>161</v>
+      </c>
+      <c r="E791" t="s">
+        <v>19</v>
+      </c>
+      <c r="F791" t="s">
+        <v>9</v>
+      </c>
+      <c r="G791">
+        <v>2019</v>
+      </c>
+      <c r="H791" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="792" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A792" s="4">
+        <f t="shared" si="5"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B792">
+        <v>12</v>
+      </c>
+      <c r="C792" t="s">
+        <v>8</v>
+      </c>
+      <c r="D792">
+        <v>167</v>
+      </c>
+      <c r="E792" t="s">
+        <v>19</v>
+      </c>
+      <c r="F792" t="s">
+        <v>9</v>
+      </c>
+      <c r="G792">
+        <v>2019</v>
+      </c>
+      <c r="H792" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="793" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A793" s="4">
+        <f t="shared" si="5"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B793">
+        <v>24</v>
+      </c>
+      <c r="C793" t="s">
+        <v>8</v>
+      </c>
+      <c r="D793">
+        <v>178</v>
+      </c>
+      <c r="E793" t="s">
+        <v>19</v>
+      </c>
+      <c r="F793" t="s">
+        <v>9</v>
+      </c>
+      <c r="G793">
+        <v>2019</v>
+      </c>
+      <c r="H793" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="794" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A794" s="4">
+        <f t="shared" si="5"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B794">
+        <v>4</v>
+      </c>
+      <c r="C794" t="s">
+        <v>14</v>
+      </c>
+      <c r="D794">
+        <v>203</v>
+      </c>
+      <c r="E794" t="s">
+        <v>19</v>
+      </c>
+      <c r="F794" t="s">
+        <v>9</v>
+      </c>
+      <c r="G794">
+        <v>2019</v>
+      </c>
+      <c r="H794" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="795" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A795" s="4">
+        <f t="shared" si="5"/>
+        <v>1E-3</v>
+      </c>
+      <c r="B795">
+        <v>8</v>
+      </c>
+      <c r="C795" t="s">
+        <v>14</v>
+      </c>
+      <c r="D795">
+        <v>226</v>
+      </c>
+      <c r="E795" t="s">
+        <v>19</v>
+      </c>
+      <c r="F795" t="s">
+        <v>9</v>
+      </c>
+      <c r="G795">
+        <v>2019</v>
+      </c>
+      <c r="H795" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>